<commit_message>
reformat and fix results (PL) logic
</commit_message>
<xml_diff>
--- a/FullSeason5.xlsx
+++ b/FullSeason5.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10512"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ianjpeck/Documents/GitHub/sbparser/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78689B4E-A462-3549-B36B-1A22218BF116}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96E35CF5-F23C-9B40-9688-AE0C801C34A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16480" xr2:uid="{786F1597-E4AA-4248-AD9D-56520FFD76E3}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1573" uniqueCount="318">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1566" uniqueCount="323">
   <si>
     <t>Month 1</t>
   </si>
@@ -1104,24 +1104,9 @@
     <t>Toon Link, ROB, Sonic, Pikachu, Diddy Kong</t>
   </si>
   <si>
-    <t>PL</t>
-  </si>
-  <si>
-    <t>Pikachu 10% Handicap from Tag Team Match</t>
-  </si>
-  <si>
     <t>Pit, Fox, Yoshi, Mr. Game &amp; Watch, Luigi</t>
   </si>
   <si>
-    <t>PL: Self Destruct</t>
-  </si>
-  <si>
-    <t>3,5,2,4,1</t>
-  </si>
-  <si>
-    <t>PL 80%</t>
-  </si>
-  <si>
     <t>Need to outlaw hammers</t>
   </si>
   <si>
@@ -1149,7 +1134,37 @@
     <t>Final Destination Tournament</t>
   </si>
   <si>
-    <t>#1 contender Tag+A827</t>
+    <t>Brawl Scramble</t>
+  </si>
+  <si>
+    <t>Sonic (PL)</t>
+  </si>
+  <si>
+    <t>ROB (PL)</t>
+  </si>
+  <si>
+    <t>Toon Link (PL)</t>
+  </si>
+  <si>
+    <t>Pikachu (PL)</t>
+  </si>
+  <si>
+    <t>Melee Scramble</t>
+  </si>
+  <si>
+    <t>Yoshi (PL)</t>
+  </si>
+  <si>
+    <t>Mr. Game &amp; Watch - W (PL)</t>
+  </si>
+  <si>
+    <t>Mr. Game &amp; Watch (PL)</t>
+  </si>
+  <si>
+    <t>Pit - W (PL)</t>
+  </si>
+  <si>
+    <t>Pikachu 10% Handicap</t>
   </si>
 </sst>
 </file>
@@ -1326,7 +1341,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1456,9 +1471,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -3617,7 +3629,7 @@
         <v>1</v>
       </c>
       <c r="C143" s="5" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="D143" s="6"/>
       <c r="E143" s="6"/>
@@ -4855,7 +4867,7 @@
         <v>1</v>
       </c>
       <c r="C236" s="5" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="D236" s="6"/>
       <c r="E236" s="6"/>
@@ -5923,7 +5935,7 @@
         <v>14</v>
       </c>
       <c r="C317" s="9" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="D317" s="10"/>
       <c r="E317" s="10"/>
@@ -7183,7 +7195,7 @@
         <v>14</v>
       </c>
       <c r="C410" s="9" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="D410" s="10"/>
       <c r="E410" s="10"/>
@@ -10016,17 +10028,17 @@
     <row r="626" spans="1:6" ht="21" x14ac:dyDescent="0.25">
       <c r="A626" s="12"/>
       <c r="B626" s="13" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="C626" s="14" t="s">
         <v>15</v>
       </c>
       <c r="D626" s="15"/>
       <c r="E626" s="15" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="F626" s="15" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
     </row>
     <row r="627" spans="1:6" x14ac:dyDescent="0.2">
@@ -10242,16 +10254,16 @@
       <c r="F641" s="15"/>
     </row>
     <row r="642" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A642" s="54"/>
-      <c r="B642" s="54"/>
-      <c r="C642" s="55">
-        <v>0</v>
-      </c>
-      <c r="D642" s="55">
-        <v>1</v>
-      </c>
-      <c r="E642" s="55"/>
-      <c r="F642" s="55"/>
+      <c r="A642" s="53"/>
+      <c r="B642" s="53"/>
+      <c r="C642" s="54">
+        <v>0</v>
+      </c>
+      <c r="D642" s="54">
+        <v>1</v>
+      </c>
+      <c r="E642" s="54"/>
+      <c r="F642" s="54"/>
     </row>
     <row r="643" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A643" s="12" t="s">
@@ -10354,16 +10366,16 @@
       <c r="F649" s="12"/>
     </row>
     <row r="650" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A650" s="54"/>
-      <c r="B650" s="54"/>
-      <c r="C650" s="54">
-        <v>0</v>
-      </c>
-      <c r="D650" s="54">
-        <v>1</v>
-      </c>
-      <c r="E650" s="54"/>
-      <c r="F650" s="54"/>
+      <c r="A650" s="53"/>
+      <c r="B650" s="53"/>
+      <c r="C650" s="53">
+        <v>0</v>
+      </c>
+      <c r="D650" s="53">
+        <v>1</v>
+      </c>
+      <c r="E650" s="53"/>
+      <c r="F650" s="53"/>
     </row>
     <row r="651" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A651" s="12" t="s">
@@ -10410,16 +10422,16 @@
       <c r="F653" s="12"/>
     </row>
     <row r="654" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A654" s="54"/>
-      <c r="B654" s="54"/>
-      <c r="C654" s="54">
-        <v>0</v>
-      </c>
-      <c r="D654" s="54">
-        <v>1</v>
-      </c>
-      <c r="E654" s="54"/>
-      <c r="F654" s="54"/>
+      <c r="A654" s="53"/>
+      <c r="B654" s="53"/>
+      <c r="C654" s="53">
+        <v>0</v>
+      </c>
+      <c r="D654" s="53">
+        <v>1</v>
+      </c>
+      <c r="E654" s="53"/>
+      <c r="F654" s="53"/>
     </row>
     <row r="655" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A655" s="12" t="s">
@@ -10634,7 +10646,7 @@
       <c r="F669" s="26"/>
     </row>
     <row r="670" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A670" s="56"/>
+      <c r="A670" s="55"/>
       <c r="B670" s="26"/>
       <c r="C670" s="26">
         <v>0</v>
@@ -11357,7 +11369,7 @@
         <v>14</v>
       </c>
       <c r="C725" s="9" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="D725" s="10"/>
       <c r="E725" s="10"/>
@@ -12263,7 +12275,7 @@
         <v>255</v>
       </c>
       <c r="C790" s="40" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="D790" s="41"/>
       <c r="E790" s="41"/>
@@ -12887,7 +12899,7 @@
         <v>255</v>
       </c>
       <c r="C838" s="40" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="D838" s="41"/>
       <c r="E838" s="41"/>
@@ -13309,7 +13321,7 @@
         <v>1</v>
       </c>
       <c r="C869" s="36" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="D869" s="37"/>
       <c r="E869" s="37"/>
@@ -13625,7 +13637,7 @@
         <v>1</v>
       </c>
       <c r="C893" s="36" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="D893" s="37"/>
       <c r="E893" s="37"/>
@@ -13855,7 +13867,7 @@
     </row>
     <row r="911" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A911" s="38" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="B911" s="38"/>
       <c r="C911" s="41">
@@ -14813,7 +14825,7 @@
         <v>1</v>
       </c>
       <c r="C984" s="36" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="D984" s="37"/>
       <c r="E984" s="37"/>
@@ -16217,7 +16229,7 @@
     </row>
     <row r="1091" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1091" s="38" t="s">
-        <v>317</v>
+        <v>265</v>
       </c>
       <c r="B1091" s="38">
         <v>3</v>
@@ -16799,7 +16811,7 @@
     </row>
     <row r="1133" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1133" s="44" t="s">
-        <v>78</v>
+        <v>312</v>
       </c>
       <c r="B1133" s="44">
         <v>6</v>
@@ -16808,7 +16820,7 @@
         <v>121</v>
       </c>
       <c r="D1133" s="47" t="s">
-        <v>107</v>
+        <v>313</v>
       </c>
       <c r="E1133" s="47"/>
       <c r="F1133" s="47"/>
@@ -16818,11 +16830,11 @@
         <v>301</v>
       </c>
       <c r="B1134" s="44"/>
-      <c r="C1134" s="53">
-        <v>0.8</v>
-      </c>
-      <c r="D1134" s="47" t="s">
-        <v>302</v>
+      <c r="C1134" s="47">
+        <v>1</v>
+      </c>
+      <c r="D1134" s="47">
+        <v>0</v>
       </c>
       <c r="E1134" s="47"/>
       <c r="F1134" s="47"/>
@@ -16833,7 +16845,7 @@
         <v>7</v>
       </c>
       <c r="C1135" s="47" t="s">
-        <v>3</v>
+        <v>314</v>
       </c>
       <c r="D1135" s="47" t="s">
         <v>9</v>
@@ -16844,24 +16856,24 @@
     <row r="1136" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1136" s="44"/>
       <c r="B1136" s="44"/>
-      <c r="C1136" s="47" t="s">
-        <v>302</v>
-      </c>
-      <c r="D1136" s="53">
-        <v>0.3</v>
+      <c r="C1136" s="47">
+        <v>0</v>
+      </c>
+      <c r="D1136" s="47">
+        <v>1</v>
       </c>
       <c r="E1136" s="47"/>
       <c r="F1136" s="47"/>
     </row>
     <row r="1137" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1137" s="44" t="s">
-        <v>303</v>
+        <v>322</v>
       </c>
       <c r="B1137" s="44">
         <v>8</v>
       </c>
       <c r="C1137" s="47" t="s">
-        <v>114</v>
+        <v>315</v>
       </c>
       <c r="D1137" s="47" t="s">
         <v>41</v>
@@ -16872,22 +16884,24 @@
     <row r="1138" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1138" s="44"/>
       <c r="B1138" s="44"/>
-      <c r="C1138" s="47" t="s">
-        <v>302</v>
-      </c>
-      <c r="D1138" s="53">
-        <v>0.6</v>
+      <c r="C1138" s="47">
+        <v>0</v>
+      </c>
+      <c r="D1138" s="47">
+        <v>1</v>
       </c>
       <c r="E1138" s="47"/>
       <c r="F1138" s="47"/>
     </row>
     <row r="1139" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1139" s="44"/>
+      <c r="A1139" s="44" t="s">
+        <v>78</v>
+      </c>
       <c r="B1139" s="44">
         <v>9</v>
       </c>
       <c r="C1139" s="47" t="s">
-        <v>109</v>
+        <v>316</v>
       </c>
       <c r="D1139" s="47" t="s">
         <v>33</v>
@@ -16898,22 +16912,24 @@
     <row r="1140" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1140" s="44"/>
       <c r="B1140" s="44"/>
-      <c r="C1140" s="47" t="s">
-        <v>302</v>
-      </c>
-      <c r="D1140" s="47"/>
+      <c r="C1140" s="47">
+        <v>0</v>
+      </c>
+      <c r="D1140" s="47">
+        <v>1</v>
+      </c>
       <c r="E1140" s="47"/>
       <c r="F1140" s="47"/>
     </row>
     <row r="1141" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1141" s="44" t="s">
-        <v>75</v>
+        <v>317</v>
       </c>
       <c r="B1141" s="44">
         <v>10</v>
       </c>
       <c r="C1141" s="47" t="s">
-        <v>26</v>
+        <v>318</v>
       </c>
       <c r="D1141" s="47" t="s">
         <v>17</v>
@@ -16923,27 +16939,25 @@
     </row>
     <row r="1142" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1142" s="49" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="B1142" s="44"/>
-      <c r="C1142" s="47" t="s">
-        <v>305</v>
-      </c>
-      <c r="D1142" s="53">
-        <v>0</v>
+      <c r="C1142" s="47">
+        <v>0</v>
+      </c>
+      <c r="D1142" s="47">
+        <v>1</v>
       </c>
       <c r="E1142" s="47"/>
       <c r="F1142" s="47"/>
     </row>
     <row r="1143" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1143" s="44" t="s">
-        <v>306</v>
-      </c>
+      <c r="A1143" s="44"/>
       <c r="B1143" s="44">
         <v>11</v>
       </c>
       <c r="C1143" s="47" t="s">
-        <v>17</v>
+        <v>319</v>
       </c>
       <c r="D1143" s="47" t="s">
         <v>43</v>
@@ -16954,10 +16968,12 @@
     <row r="1144" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1144" s="44"/>
       <c r="B1144" s="44"/>
-      <c r="C1144" s="47" t="s">
-        <v>307</v>
-      </c>
-      <c r="D1144" s="47"/>
+      <c r="C1144" s="47">
+        <v>1</v>
+      </c>
+      <c r="D1144" s="47">
+        <v>0</v>
+      </c>
       <c r="E1144" s="47"/>
       <c r="F1144" s="47"/>
     </row>
@@ -16967,7 +16983,7 @@
         <v>12</v>
       </c>
       <c r="C1145" s="47" t="s">
-        <v>110</v>
+        <v>320</v>
       </c>
       <c r="D1145" s="47" t="s">
         <v>27</v>
@@ -16978,22 +16994,24 @@
     <row r="1146" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1146" s="44"/>
       <c r="B1146" s="44"/>
-      <c r="C1146" s="47" t="s">
-        <v>302</v>
-      </c>
-      <c r="D1146" s="53">
-        <v>0</v>
+      <c r="C1146" s="47">
+        <v>0</v>
+      </c>
+      <c r="D1146" s="47">
+        <v>1</v>
       </c>
       <c r="E1146" s="47"/>
       <c r="F1146" s="47"/>
     </row>
     <row r="1147" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1147" s="44"/>
+      <c r="A1147" s="44" t="s">
+        <v>75</v>
+      </c>
       <c r="B1147" s="44">
         <v>13</v>
       </c>
       <c r="C1147" s="47" t="s">
-        <v>27</v>
+        <v>321</v>
       </c>
       <c r="D1147" s="47" t="s">
         <v>83</v>
@@ -17004,10 +17022,12 @@
     <row r="1148" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1148" s="44"/>
       <c r="B1148" s="44"/>
-      <c r="C1148" s="47" t="s">
-        <v>302</v>
-      </c>
-      <c r="D1148" s="47"/>
+      <c r="C1148" s="47">
+        <v>1</v>
+      </c>
+      <c r="D1148" s="47">
+        <v>0</v>
+      </c>
       <c r="E1148" s="47"/>
       <c r="F1148" s="47"/>
     </row>

</xml_diff>

<commit_message>
rerun files and update todo
</commit_message>
<xml_diff>
--- a/FullSeason5.xlsx
+++ b/FullSeason5.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ianjpeck/Documents/GitHub/sbparser/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{835D1831-37CA-F247-9A7C-1053CF574247}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A10C61B-7DBC-6446-978B-42E710A2B4CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{C96D0F46-2D53-AF4F-A06C-8FE540EC6340}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16500" xr2:uid="{C96D0F46-2D53-AF4F-A06C-8FE540EC6340}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1572" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1572" uniqueCount="324">
   <si>
     <t>Month 1</t>
   </si>
@@ -1081,9 +1081,6 @@
   </si>
   <si>
     <t>Coin Match, 1st time champion has lost at Championship Cruise</t>
-  </si>
-  <si>
-    <t>Hardcore Chamionship</t>
   </si>
   <si>
     <t>Wolf 140% Handicap</t>
@@ -15574,7 +15571,7 @@
     </row>
     <row r="1038" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1038" s="46" t="s">
-        <v>295</v>
+        <v>72</v>
       </c>
       <c r="B1038" s="46">
         <v>4</v>
@@ -15622,7 +15619,7 @@
     </row>
     <row r="1041" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1041" s="46" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B1041" s="46"/>
       <c r="C1041" s="49">
@@ -15684,7 +15681,7 @@
     </row>
     <row r="1045" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1045" s="51" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B1045" s="46"/>
       <c r="C1045" s="49">
@@ -15698,7 +15695,7 @@
     </row>
     <row r="1046" spans="1:6" ht="25" x14ac:dyDescent="0.25">
       <c r="A1046" s="33" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B1046" s="33"/>
       <c r="C1046" s="34"/>
@@ -15934,7 +15931,7 @@
     </row>
     <row r="1065" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1065" s="40" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B1065" s="40">
         <v>3</v>
@@ -16190,7 +16187,7 @@
     </row>
     <row r="1085" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1085" s="40" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B1085" s="40">
         <v>1</v>
@@ -16348,7 +16345,7 @@
         <v>1</v>
       </c>
       <c r="C1096" s="38" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D1096" s="39"/>
       <c r="E1096" s="39"/>
@@ -16504,7 +16501,7 @@
         <v>262</v>
       </c>
       <c r="C1108" s="42" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D1108" s="43"/>
       <c r="E1108" s="43"/>
@@ -16580,7 +16577,7 @@
     </row>
     <row r="1114" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1114" s="40" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B1114" s="40"/>
       <c r="C1114" s="43">
@@ -16659,10 +16656,10 @@
     <row r="1120" spans="1:6" ht="22" x14ac:dyDescent="0.3">
       <c r="A1120" s="46"/>
       <c r="B1120" s="47" t="s">
+        <v>303</v>
+      </c>
+      <c r="C1120" s="48" t="s">
         <v>304</v>
-      </c>
-      <c r="C1120" s="48" t="s">
-        <v>305</v>
       </c>
       <c r="D1120" s="49"/>
       <c r="E1120" s="49"/>
@@ -16686,7 +16683,7 @@
     </row>
     <row r="1122" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1122" s="46" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B1122" s="46"/>
       <c r="C1122" s="49">
@@ -16716,7 +16713,7 @@
     </row>
     <row r="1124" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1124" s="46" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B1124" s="46"/>
       <c r="C1124" s="49">
@@ -16826,7 +16823,7 @@
     </row>
     <row r="1131" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1131" s="46" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B1131" s="46">
         <v>6</v>
@@ -16835,14 +16832,14 @@
         <v>122</v>
       </c>
       <c r="D1131" s="49" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="E1131" s="49"/>
       <c r="F1131" s="49"/>
     </row>
     <row r="1132" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1132" s="46" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B1132" s="46"/>
       <c r="C1132" s="49">
@@ -16856,13 +16853,13 @@
     </row>
     <row r="1133" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1133" s="51" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B1133" s="46">
         <v>7</v>
       </c>
       <c r="C1133" s="49" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="D1133" s="49" t="s">
         <v>9</v>
@@ -16884,13 +16881,13 @@
     </row>
     <row r="1135" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1135" s="46" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B1135" s="46">
         <v>8</v>
       </c>
       <c r="C1135" s="49" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D1135" s="49" t="s">
         <v>41</v>
@@ -16912,13 +16909,13 @@
     </row>
     <row r="1137" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1137" s="46" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B1137" s="46">
         <v>10</v>
       </c>
       <c r="C1137" s="49" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D1137" s="49" t="s">
         <v>33</v>
@@ -16940,13 +16937,13 @@
     </row>
     <row r="1139" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1139" s="46" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B1139" s="46">
         <v>11</v>
       </c>
       <c r="C1139" s="49" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D1139" s="49" t="s">
         <v>17</v>
@@ -16956,7 +16953,7 @@
     </row>
     <row r="1140" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1140" s="51" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B1140" s="46"/>
       <c r="C1140" s="49">
@@ -16970,13 +16967,13 @@
     </row>
     <row r="1141" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1141" s="46" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B1141" s="46">
         <v>12</v>
       </c>
       <c r="C1141" s="49" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D1141" s="49" t="s">
         <v>43</v>
@@ -16998,13 +16995,13 @@
     </row>
     <row r="1143" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1143" s="46" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B1143" s="46">
         <v>13</v>
       </c>
       <c r="C1143" s="49" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D1143" s="49" t="s">
         <v>27</v>
@@ -17026,13 +17023,13 @@
     </row>
     <row r="1145" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1145" s="46" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B1145" s="46">
         <v>14</v>
       </c>
       <c r="C1145" s="49" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="D1145" s="49" t="s">
         <v>83</v>

</xml_diff>